<commit_message>
Compiled several sources to FR-truth Apples in Alabama as an example.
</commit_message>
<xml_diff>
--- a/data/truth_states/State-Truths.xlsx
+++ b/data/truth_states/State-Truths.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chigham\Documents\forkranger-us-regions\data\truth_states\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06D9B005-033D-4398-8F43-E764AA24643A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9843BF61-D030-446A-B85C-A7794FCFFE3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_Seasonal-Products" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="106">
   <si>
     <t>Potato</t>
   </si>
@@ -227,13 +227,130 @@
   </si>
   <si>
     <t>Peppers</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Source Link</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>June</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>August</t>
+  </si>
+  <si>
+    <t>September</t>
+  </si>
+  <si>
+    <t>October</t>
+  </si>
+  <si>
+    <t>November</t>
+  </si>
+  <si>
+    <t>December</t>
+  </si>
+  <si>
+    <t>Starting Now</t>
+  </si>
+  <si>
+    <t>Prime Time</t>
+  </si>
+  <si>
+    <t>Last Chance</t>
+  </si>
+  <si>
+    <t>http://www.fma.alabama.gov/avail_chart.htm</t>
+  </si>
+  <si>
+    <t>Seasonal Food Guide</t>
+  </si>
+  <si>
+    <t>https://www.seasonalfoodguide.org/state/alabama</t>
+  </si>
+  <si>
+    <t>https://farmflavor.com/alabama/whats-growing-alabama-produce-calendar/</t>
+  </si>
+  <si>
+    <t>Farm Flavor</t>
+  </si>
+  <si>
+    <t>State - Availability Chart (2004)</t>
+  </si>
+  <si>
+    <t>Fork Ranger</t>
+  </si>
+  <si>
+    <t>Attachment Link (Github)</t>
+  </si>
+  <si>
+    <t>https://github.com/chigham/forkranger-us-regions/blob/main/sources/states/SE_Alabama%20(2004).gif</t>
+  </si>
+  <si>
+    <t>https://github.com/chigham/forkranger-us-regions/blob/main/sources/Farm-Flavor/Alabama-scaled.jpg</t>
+  </si>
+  <si>
+    <t>https://github.com/chigham/forkranger-us-regions/blob/main/sources/Seasonal%20Food%20Guide/Alabama-apples.jpg</t>
+  </si>
+  <si>
+    <t>Alabama Farm to School (2019)</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>May Be Stored</t>
+  </si>
+  <si>
+    <t>https://alabamafarmtoece.org/wp-content/uploads/2022/04/ALSeasonal-Produce-Guide.pdf</t>
+  </si>
+  <si>
+    <t>https://github.com/chigham/forkranger-us-regions/blob/main/sources/states/SE_Alabama%20(2022)%20(Farm%20to%20School).pdf</t>
+  </si>
+  <si>
+    <t>? Great From Storage</t>
+  </si>
+  <si>
+    <t>https://acl.gov/sites/default/files/nutrition/SeasonalProduceChartByRegion.pdf; https://www.farmersalmanac.com/calendar/fruits-vegetables-season</t>
+  </si>
+  <si>
+    <t>https://github.com/chigham/forkranger-us-regions/blob/main/sources/SeasonalProduceChartByRegion.pdf</t>
+  </si>
+  <si>
+    <t>Generalized 3-month season/region data, applied to state</t>
+  </si>
+  <si>
+    <t>US Dept of HHS - Regional Seasonality (Derived from Farmers Almanac)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -248,8 +365,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -262,8 +385,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -271,16 +400,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -897,9 +1038,538 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:Q64"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" t="s">
+        <v>76</v>
+      </c>
+      <c r="J1" t="s">
+        <v>77</v>
+      </c>
+      <c r="K1" t="s">
+        <v>78</v>
+      </c>
+      <c r="L1" t="s">
+        <v>79</v>
+      </c>
+      <c r="M1" t="s">
+        <v>80</v>
+      </c>
+      <c r="N1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O1" t="s">
+        <v>69</v>
+      </c>
+      <c r="P1" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>86</v>
+      </c>
+      <c r="I3" t="s">
+        <v>82</v>
+      </c>
+      <c r="J3" t="s">
+        <v>83</v>
+      </c>
+      <c r="K3" t="s">
+        <v>83</v>
+      </c>
+      <c r="L3" t="s">
+        <v>84</v>
+      </c>
+      <c r="O3" t="s">
+        <v>87</v>
+      </c>
+      <c r="P3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>90</v>
+      </c>
+      <c r="I4" t="s">
+        <v>82</v>
+      </c>
+      <c r="J4" t="s">
+        <v>83</v>
+      </c>
+      <c r="K4" t="s">
+        <v>83</v>
+      </c>
+      <c r="L4" t="s">
+        <v>83</v>
+      </c>
+      <c r="M4" t="s">
+        <v>84</v>
+      </c>
+      <c r="O4" t="s">
+        <v>85</v>
+      </c>
+      <c r="P4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E5" t="s">
+        <v>101</v>
+      </c>
+      <c r="F5" t="s">
+        <v>101</v>
+      </c>
+      <c r="G5" t="s">
+        <v>101</v>
+      </c>
+      <c r="H5" t="s">
+        <v>101</v>
+      </c>
+      <c r="I5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J5" t="s">
+        <v>101</v>
+      </c>
+      <c r="K5" t="s">
+        <v>82</v>
+      </c>
+      <c r="L5" t="s">
+        <v>83</v>
+      </c>
+      <c r="M5" t="s">
+        <v>84</v>
+      </c>
+      <c r="N5" t="s">
+        <v>101</v>
+      </c>
+      <c r="O5" t="s">
+        <v>99</v>
+      </c>
+      <c r="P5" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>89</v>
+      </c>
+      <c r="I6" t="s">
+        <v>82</v>
+      </c>
+      <c r="J6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K6" t="s">
+        <v>83</v>
+      </c>
+      <c r="L6" t="s">
+        <v>84</v>
+      </c>
+      <c r="O6" t="s">
+        <v>88</v>
+      </c>
+      <c r="P6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>105</v>
+      </c>
+      <c r="H7" t="s">
+        <v>83</v>
+      </c>
+      <c r="I7" t="s">
+        <v>83</v>
+      </c>
+      <c r="J7" t="s">
+        <v>83</v>
+      </c>
+      <c r="O7" t="s">
+        <v>102</v>
+      </c>
+      <c r="P7" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A63" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>